<commit_message>
update retention and HTE analyses, md content
</commit_message>
<xml_diff>
--- a/results/ate_evalue_confounder_benchmarks_survey.xlsx
+++ b/results/ate_evalue_confounder_benchmarks_survey.xlsx
@@ -475,13 +475,13 @@
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.392</v>
+        <v>-0.388</v>
       </c>
       <c r="E2" t="n">
-        <v>1.4286</v>
+        <v>1.4234</v>
       </c>
       <c r="F2" t="n">
-        <v>2.21</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="3">
@@ -499,13 +499,13 @@
         <v>2</v>
       </c>
       <c r="D3" t="n">
-        <v>0.368</v>
+        <v>0.369</v>
       </c>
       <c r="E3" t="n">
-        <v>1.3978</v>
+        <v>1.399</v>
       </c>
       <c r="F3" t="n">
-        <v>2.14</v>
+        <v>2.15</v>
       </c>
     </row>
     <row r="4">
@@ -523,13 +523,13 @@
         <v>3</v>
       </c>
       <c r="D4" t="n">
-        <v>0.351</v>
+        <v>0.35</v>
       </c>
       <c r="E4" t="n">
-        <v>1.3763</v>
+        <v>1.3751</v>
       </c>
       <c r="F4" t="n">
-        <v>2.1</v>
+        <v>2.09</v>
       </c>
     </row>
     <row r="5">
@@ -547,13 +547,13 @@
         <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.392</v>
+        <v>-0.388</v>
       </c>
       <c r="E5" t="n">
-        <v>1.4286</v>
+        <v>1.4234</v>
       </c>
       <c r="F5" t="n">
-        <v>2.21</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="6">
@@ -571,13 +571,13 @@
         <v>2</v>
       </c>
       <c r="D6" t="n">
-        <v>0.368</v>
+        <v>0.369</v>
       </c>
       <c r="E6" t="n">
-        <v>1.3978</v>
+        <v>1.399</v>
       </c>
       <c r="F6" t="n">
-        <v>2.14</v>
+        <v>2.15</v>
       </c>
     </row>
     <row r="7">
@@ -595,13 +595,13 @@
         <v>3</v>
       </c>
       <c r="D7" t="n">
-        <v>0.351</v>
+        <v>0.35</v>
       </c>
       <c r="E7" t="n">
-        <v>1.3763</v>
+        <v>1.3751</v>
       </c>
       <c r="F7" t="n">
-        <v>2.1</v>
+        <v>2.09</v>
       </c>
     </row>
     <row r="8">
@@ -619,13 +619,13 @@
         <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.392</v>
+        <v>-0.388</v>
       </c>
       <c r="E8" t="n">
-        <v>1.4286</v>
+        <v>1.4234</v>
       </c>
       <c r="F8" t="n">
-        <v>2.21</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="9">
@@ -643,13 +643,13 @@
         <v>2</v>
       </c>
       <c r="D9" t="n">
-        <v>0.368</v>
+        <v>0.369</v>
       </c>
       <c r="E9" t="n">
-        <v>1.3978</v>
+        <v>1.399</v>
       </c>
       <c r="F9" t="n">
-        <v>2.14</v>
+        <v>2.15</v>
       </c>
     </row>
     <row r="10">
@@ -667,13 +667,13 @@
         <v>3</v>
       </c>
       <c r="D10" t="n">
-        <v>0.351</v>
+        <v>0.35</v>
       </c>
       <c r="E10" t="n">
-        <v>1.3763</v>
+        <v>1.3751</v>
       </c>
       <c r="F10" t="n">
-        <v>2.1</v>
+        <v>2.09</v>
       </c>
     </row>
   </sheetData>

</xml_diff>